<commit_message>
Scope OR TW extract rows so MP lookups hit a single rate.
Fill CC bands and state-specific RTO lists on the three overlapping New(1+5) rows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/masters/grid_import_split/OR_grid_26-27.xlsx
+++ b/masters/grid_import_split/OR_grid_26-27.xlsx
@@ -801,17 +801,6 @@
           <t>31-03-2027</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
         <v>2.01</v>
       </c>
@@ -833,17 +822,6 @@
           <t>Madhya Pradesh / Uttar Pradesh / Tamil Nadu — excluded-state bucket</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
         <v>0.2</v>
       </c>
@@ -852,33 +830,6 @@
           <t>NET (OD+TP)</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr">
         <is>
           <t>7.grid_Oriental_Motor_2026-27.xlsx</t>
@@ -1292,34 +1243,9 @@
           <t>0 (brand new) — assumed</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
       <c r="T2" t="n">
         <v>6</v>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
         <v>0.2</v>
       </c>
@@ -1328,33 +1254,6 @@
           <t>NET (OD+TP), brand new</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
-      <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr">
         <is>
           <t>7.grid_Oriental_Motor_2026-27.xlsx</t>
@@ -1768,40 +1667,32 @@
           <t>0 (brand new)</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>350</v>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
           <t>Madhya Pradesh (+ Assam) — flat-rate excluded-state bucket</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>PAN INDIA</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>MP</t>
+        </is>
+      </c>
       <c r="AB2" t="inlineStr">
         <is>
           <t>~689 MP-resolved policies (most are typical ≤350cc commuter bikes)</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
         <v>0.05</v>
       </c>
@@ -1810,32 +1701,9 @@
           <t>NET (OD+TP combined)</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
+      <c r="AQ2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="BM2" t="n">
         <v>689</v>
       </c>
@@ -1901,40 +1769,32 @@
           <t>0 (brand new)</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>150</v>
+      </c>
+      <c r="P3" t="n">
+        <v>350</v>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
           <t>Chhattisgarh — flat-rate excluded-state bucket (150-350cc band only)</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>CG-04</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
       <c r="AB3" t="inlineStr">
         <is>
           <t>~98 CG-resolved policies</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="n">
         <v>0.05</v>
       </c>
@@ -1943,32 +1803,9 @@
           <t>NET (OD+TP combined)</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
-      <c r="BE3" t="inlineStr"/>
-      <c r="BF3" t="inlineStr"/>
-      <c r="BG3" t="inlineStr"/>
-      <c r="BH3" t="inlineStr"/>
-      <c r="BI3" t="inlineStr"/>
-      <c r="BJ3" t="inlineStr"/>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="inlineStr"/>
+      <c r="AQ3" t="n">
+        <v>0.05</v>
+      </c>
       <c r="BM3" t="n">
         <v>98</v>
       </c>
@@ -2034,40 +1871,32 @@
           <t>0 (brand new)</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>150</v>
+      </c>
       <c r="Y4" t="inlineStr">
         <is>
           <t>Uttar Pradesh — not an excluded state (discount-tiered)</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>UP-32</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
       <c r="AB4" t="inlineStr">
         <is>
           <t>~32 UP-resolved policies</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="n">
         <v>0.3</v>
       </c>
@@ -2084,30 +1913,9 @@
           <t>TP</t>
         </is>
       </c>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="inlineStr"/>
-      <c r="BA4" t="inlineStr"/>
-      <c r="BB4" t="inlineStr"/>
-      <c r="BC4" t="inlineStr"/>
-      <c r="BD4" t="inlineStr"/>
-      <c r="BE4" t="inlineStr"/>
-      <c r="BF4" t="inlineStr"/>
-      <c r="BG4" t="inlineStr"/>
-      <c r="BH4" t="inlineStr"/>
-      <c r="BI4" t="inlineStr"/>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="inlineStr"/>
+      <c r="AQ4" t="n">
+        <v>0.3</v>
+      </c>
       <c r="BM4" t="n">
         <v>32</v>
       </c>

</xml_diff>